<commit_message>
Adiciona campo "codAgl" na tabela de plano  de contas  e atualiza planilha de contas
</commit_message>
<xml_diff>
--- a/upload/plano_conta.xlsx
+++ b/upload/plano_conta.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/597695ca0a7eda65/Documentos/Inovare/Netsuite/layout de importação por planilha/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/597695ca0a7eda65/Documentos/Inovare/Netsuite/doc-netsuite/upload/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="82" documentId="8_{9DFFF064-0DFB-4EB0-9596-DD8710511CE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{73E58AAA-F145-4AE6-BA7A-219FD793A825}"/>
+  <xr:revisionPtr revIDLastSave="84" documentId="8_{9DFFF064-0DFB-4EB0-9596-DD8710511CE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E45CB6C5-2F62-4BFC-A301-89AC4F572D7C}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{66AC0E31-F421-4071-93E6-EA0F1765406F}"/>
+    <workbookView xWindow="0" yWindow="24" windowWidth="23040" windowHeight="12216" xr2:uid="{66AC0E31-F421-4071-93E6-EA0F1765406F}"/>
   </bookViews>
   <sheets>
     <sheet name="dados" sheetId="1" r:id="rId1"/>
@@ -50,6 +50,7 @@
     <author>tc={6EDCEB8B-3580-49C7-BA05-C567FF721719}</author>
     <author>tc={4B445772-1894-4B2C-8BDB-053E90A8D281}</author>
     <author>tc={5F0858C9-BC9A-458A-859A-D06266E20794}</author>
+    <author>tc={416C3512-5626-46F6-A9ED-09C2CF24976F}</author>
   </authors>
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0" xr:uid="{C138AF36-D45A-4766-B3A3-0F7F3700C519}">
@@ -146,6 +147,14 @@
 Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
 Comentário:
     Campo opcional que só deve ser preenchido se for enviar plano referencial por centro de custos</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="12" shapeId="0" xr:uid="{416C3512-5626-46F6-A9ED-09C2CF24976F}">
+      <text>
+        <t>[Comentário encadeado]
+Sua versão do Excel permite que você leia este comentário encadeado, no entanto, as edições serão removidas se o arquivo for aberto em uma versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
+Comentário:
+    Opcional, só deve ser utilizado se quiser personalizar demonstração contábil da ECD. Aqui deve ser enviado o código de aglutinação que conta irá utilizar para montar demonstrações contábeis da ECD.</t>
       </text>
     </comment>
   </commentList>
@@ -153,7 +162,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
   <si>
     <t>cnpjEmpr</t>
   </si>
@@ -213,6 +222,9 @@
   </si>
   <si>
     <t>codCentroCusto</t>
+  </si>
+  <si>
+    <t>codAgl</t>
   </si>
 </sst>
 </file>
@@ -262,13 +274,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -645,18 +655,20 @@
   <threadedComment ref="L1" dT="2026-03-23T18:16:36.30" personId="{FAFA3D93-AFA3-4FD9-A670-ED0A9643D14B}" id="{5F0858C9-BC9A-458A-859A-D06266E20794}">
     <text>Campo opcional que só deve ser preenchido se for enviar plano referencial por centro de custos</text>
   </threadedComment>
+  <threadedComment ref="M1" dT="2026-04-12T14:59:02.34" personId="{FAFA3D93-AFA3-4FD9-A670-ED0A9643D14B}" id="{416C3512-5626-46F6-A9ED-09C2CF24976F}">
+    <text>Opcional, só deve ser utilizado se quiser personalizar demonstração contábil da ECD. Aqui deve ser enviado o código de aglutinação que conta irá utilizar para montar demonstrações contábeis da ECD.</text>
+  </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66BD541C-B0A8-45D0-83BF-E03A8CD2EF40}">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.109375" style="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.33203125" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="8.88671875" style="3"/>
-    <col min="5" max="5" width="8.88671875" style="4"/>
     <col min="6" max="6" width="8.88671875" style="3"/>
     <col min="7" max="7" width="10.44140625" style="3" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.44140625" style="3" customWidth="1"/>
@@ -665,7 +677,7 @@
     <col min="12" max="12" width="14.77734375" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -678,7 +690,7 @@
       <c r="D1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="F1" s="2" t="s">
@@ -702,8 +714,11 @@
       <c r="L1" s="2" t="s">
         <v>19</v>
       </c>
+      <c r="M1" s="2" t="s">
+        <v>20</v>
+      </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>2</v>
       </c>
@@ -716,7 +731,7 @@
       <c r="D2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2">
         <v>1</v>
       </c>
       <c r="F2" s="3" t="s">

</xml_diff>